<commit_message>
fix(scripts): sửa lời gọi read_df khi xuất công nợ, ghi ngày dạng yyyy-MM-dd (#18)
</commit_message>
<xml_diff>
--- a/data/export/si_so_lop.xlsx
+++ b/data/export/si_so_lop.xlsx
@@ -523,11 +523,15 @@
           <t>Trần Khánh Mai</t>
         </is>
       </c>
-      <c r="F2" s="1" t="n">
-        <v>45698</v>
-      </c>
-      <c r="G2" s="1" t="n">
-        <v>45784</v>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2025-02-10</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2025-05-07</t>
+        </is>
       </c>
       <c r="H2" t="n">
         <v>19</v>
@@ -575,11 +579,15 @@
           <t>Lê Thanh Yến</t>
         </is>
       </c>
-      <c r="F3" s="1" t="n">
-        <v>45719</v>
-      </c>
-      <c r="G3" s="1" t="n">
-        <v>45805</v>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2025-03-03</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2025-05-28</t>
+        </is>
       </c>
       <c r="H3" t="n">
         <v>18</v>
@@ -627,11 +635,15 @@
           <t>Mai Ngọc Duyên</t>
         </is>
       </c>
-      <c r="F4" s="1" t="n">
-        <v>45833</v>
-      </c>
-      <c r="G4" s="1" t="n">
-        <v>45898</v>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2025-06-25</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2025-08-29</t>
+        </is>
       </c>
       <c r="H4" t="n">
         <v>21</v>
@@ -679,11 +691,15 @@
           <t>Lê Minh Thảo</t>
         </is>
       </c>
-      <c r="F5" s="1" t="n">
-        <v>45957</v>
-      </c>
-      <c r="G5" s="1" t="n">
-        <v>46036</v>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2025-10-27</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
       </c>
       <c r="H5" t="n">
         <v>24</v>
@@ -731,11 +747,15 @@
           <t>Trần Khánh Mai</t>
         </is>
       </c>
-      <c r="F6" s="1" t="n">
-        <v>46146</v>
-      </c>
-      <c r="G6" s="1" t="n">
-        <v>46211</v>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
       </c>
       <c r="H6" t="n">
         <v>29</v>
@@ -783,11 +803,15 @@
           <t>Mai Ngọc Duyên</t>
         </is>
       </c>
-      <c r="F7" s="1" t="n">
-        <v>46251</v>
-      </c>
-      <c r="G7" s="1" t="n">
-        <v>46335</v>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
       </c>
       <c r="H7" t="n">
         <v>27</v>
@@ -835,11 +859,15 @@
           <t>Lê Thanh Yến</t>
         </is>
       </c>
-      <c r="F8" s="1" t="n">
-        <v>46253</v>
-      </c>
-      <c r="G8" s="1" t="n">
-        <v>46358</v>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
       </c>
       <c r="H8" t="n">
         <v>20</v>
@@ -887,11 +915,15 @@
           <t>Lê Minh Thảo</t>
         </is>
       </c>
-      <c r="F9" s="1" t="n">
-        <v>46326</v>
-      </c>
-      <c r="G9" s="1" t="n">
-        <v>46425</v>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2027-02-07</t>
+        </is>
       </c>
       <c r="H9" t="n">
         <v>19</v>
@@ -939,11 +971,15 @@
           <t>Trần Khánh Mai</t>
         </is>
       </c>
-      <c r="F10" s="1" t="n">
-        <v>46347</v>
-      </c>
-      <c r="G10" s="1" t="n">
-        <v>46425</v>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-11-21</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2027-02-07</t>
+        </is>
       </c>
       <c r="H10" t="n">
         <v>12</v>
@@ -991,11 +1027,15 @@
           <t>Bùi Bảo Yến</t>
         </is>
       </c>
-      <c r="F11" s="1" t="n">
-        <v>45710</v>
-      </c>
-      <c r="G11" s="1" t="n">
-        <v>45774</v>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2025-02-22</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2025-04-27</t>
+        </is>
       </c>
       <c r="H11" t="n">
         <v>24</v>
@@ -1043,11 +1083,15 @@
           <t>Bùi Đức Nhiên</t>
         </is>
       </c>
-      <c r="F12" s="1" t="n">
-        <v>45818</v>
-      </c>
-      <c r="G12" s="1" t="n">
-        <v>45923</v>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2025-06-10</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2025-09-23</t>
+        </is>
       </c>
       <c r="H12" t="n">
         <v>17</v>
@@ -1095,11 +1139,15 @@
           <t>Hoàng Quang Quang</t>
         </is>
       </c>
-      <c r="F13" s="1" t="n">
-        <v>45843</v>
-      </c>
-      <c r="G13" s="1" t="n">
-        <v>45921</v>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2025-07-05</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2025-09-21</t>
+        </is>
       </c>
       <c r="H13" t="n">
         <v>21</v>
@@ -1147,11 +1195,15 @@
           <t>Bùi Bảo Yến</t>
         </is>
       </c>
-      <c r="F14" s="1" t="n">
-        <v>45964</v>
-      </c>
-      <c r="G14" s="1" t="n">
-        <v>46029</v>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2025-11-03</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-01-07</t>
+        </is>
       </c>
       <c r="H14" t="n">
         <v>18</v>
@@ -1199,11 +1251,15 @@
           <t>Bùi Đức Nhiên</t>
         </is>
       </c>
-      <c r="F15" s="1" t="n">
-        <v>46134</v>
-      </c>
-      <c r="G15" s="1" t="n">
-        <v>46218</v>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
       </c>
       <c r="H15" t="n">
         <v>26</v>
@@ -1251,11 +1307,15 @@
           <t>Hoàng Quang Quang</t>
         </is>
       </c>
-      <c r="F16" s="1" t="n">
-        <v>46158</v>
-      </c>
-      <c r="G16" s="1" t="n">
-        <v>46236</v>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
       </c>
       <c r="H16" t="n">
         <v>28</v>
@@ -1303,11 +1363,15 @@
           <t>Bùi Bảo Yến</t>
         </is>
       </c>
-      <c r="F17" s="1" t="n">
-        <v>46260</v>
-      </c>
-      <c r="G17" s="1" t="n">
-        <v>46330</v>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
       </c>
       <c r="H17" t="n">
         <v>26</v>
@@ -1355,11 +1419,15 @@
           <t>Bùi Đức Nhiên</t>
         </is>
       </c>
-      <c r="F18" s="1" t="n">
-        <v>46330</v>
-      </c>
-      <c r="G18" s="1" t="n">
-        <v>46409</v>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2027-01-22</t>
+        </is>
       </c>
       <c r="H18" t="n">
         <v>15</v>
@@ -1407,11 +1475,15 @@
           <t>Smith John</t>
         </is>
       </c>
-      <c r="F19" s="1" t="n">
-        <v>45714</v>
-      </c>
-      <c r="G19" s="1" t="n">
-        <v>45784</v>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2025-02-26</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2025-05-07</t>
+        </is>
       </c>
       <c r="H19" t="n">
         <v>18</v>
@@ -1459,11 +1531,15 @@
           <t>Brown Emily</t>
         </is>
       </c>
-      <c r="F20" s="1" t="n">
-        <v>45829</v>
-      </c>
-      <c r="G20" s="1" t="n">
-        <v>45907</v>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2025-06-21</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2025-09-07</t>
+        </is>
       </c>
       <c r="H20" t="n">
         <v>18</v>
@@ -1511,11 +1587,15 @@
           <t>Wilson David</t>
         </is>
       </c>
-      <c r="F21" s="1" t="n">
-        <v>45950</v>
-      </c>
-      <c r="G21" s="1" t="n">
-        <v>46050</v>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2025-10-20</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
       </c>
       <c r="H21" t="n">
         <v>20</v>
@@ -1563,11 +1643,15 @@
           <t>Smith John</t>
         </is>
       </c>
-      <c r="F22" s="1" t="n">
-        <v>45976</v>
-      </c>
-      <c r="G22" s="1" t="n">
-        <v>46054</v>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2025-11-15</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
       </c>
       <c r="H22" t="n">
         <v>19</v>
@@ -1615,11 +1699,15 @@
           <t>Brown Emily</t>
         </is>
       </c>
-      <c r="F23" s="1" t="n">
-        <v>46140</v>
-      </c>
-      <c r="G23" s="1" t="n">
-        <v>46210</v>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
       </c>
       <c r="H23" t="n">
         <v>24</v>
@@ -1667,11 +1755,15 @@
           <t>Wilson David</t>
         </is>
       </c>
-      <c r="F24" s="1" t="n">
-        <v>46249</v>
-      </c>
-      <c r="G24" s="1" t="n">
-        <v>46348</v>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2026-11-22</t>
+        </is>
       </c>
       <c r="H24" t="n">
         <v>28</v>
@@ -1719,11 +1811,15 @@
           <t>Smith John</t>
         </is>
       </c>
-      <c r="F25" s="1" t="n">
-        <v>46265</v>
-      </c>
-      <c r="G25" s="1" t="n">
-        <v>46349</v>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2026-11-23</t>
+        </is>
       </c>
       <c r="H25" t="n">
         <v>23</v>
@@ -1771,11 +1867,15 @@
           <t>Brown Emily</t>
         </is>
       </c>
-      <c r="F26" s="1" t="n">
-        <v>46336</v>
-      </c>
-      <c r="G26" s="1" t="n">
-        <v>46401</v>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2027-01-14</t>
+        </is>
       </c>
       <c r="H26" t="n">
         <v>10</v>
@@ -1817,8 +1917,8 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
   </cols>

</xml_diff>